<commit_message>
updates based on new HM model
</commit_message>
<xml_diff>
--- a/inputs/preprocessing/crosslinks_biochemical/crosslinks/crosslink_papers/zhu_2024/micos_xlinks.xlsx
+++ b/inputs/preprocessing/crosslinks_biochemical/crosslinks/crosslink_papers/zhu_2024/micos_xlinks.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,7 +457,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -466,7 +466,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>423</t>
+          <t>506</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -476,13 +476,13 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>423</t>
+          <t>516</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -491,7 +491,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>423</t>
+          <t>581</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -501,13 +501,13 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>436</t>
+          <t>581</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -516,7 +516,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>427</t>
+          <t>640</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -526,13 +526,13 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>438</t>
+          <t>640</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -541,23 +541,23 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>436</t>
+          <t>714</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MIC60</t>
+          <t>MIC10</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>438</t>
+          <t>74</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -571,18 +571,18 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MIC60</t>
+          <t>MIC19</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>121</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -591,23 +591,23 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>581</t>
+          <t>506</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MIC60</t>
+          <t>MIC19</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>581</t>
+          <t>136</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -616,23 +616,23 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>516</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MIC60</t>
+          <t>MIC19</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>130</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -641,23 +641,23 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>714</t>
+          <t>516</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MIC10</t>
+          <t>MIC19</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>136</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>506</t>
+          <t>581</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -676,22 +676,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>219</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>130</v>
+        <v>4351</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MIC60</t>
+          <t>MIC19</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>506</t>
+          <t>86</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -701,22 +701,22 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>76</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>131</v>
+        <v>4352</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MIC60</t>
+          <t>MIC19</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>119</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -726,22 +726,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>77</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>132</v>
+        <v>4353</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MIC60</t>
+          <t>MIC19</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>121</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -751,22 +751,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>165</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>133</v>
+        <v>4354</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MIC60</t>
+          <t>MIC19</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>581</t>
+          <t>121</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -776,13 +776,13 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>219</t>
+          <t>63</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>4351</v>
+        <v>4355</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>121</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -807,7 +807,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>4352</v>
+        <v>4356</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -816,7 +816,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>130</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -826,13 +826,13 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>136</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>4353</v>
+        <v>4357</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -841,7 +841,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>130</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -851,13 +851,13 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>77</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>4354</v>
+        <v>4358</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -866,7 +866,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>136</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -876,13 +876,13 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>136</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>4355</v>
+        <v>4359</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>136</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -901,13 +901,13 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>142</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>4356</v>
+        <v>4360</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>136</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -926,13 +926,13 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>165</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>4357</v>
+        <v>4361</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>136</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -951,13 +951,13 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>173</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>4358</v>
+        <v>4362</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -976,13 +976,13 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>45</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>4359</v>
+        <v>4363</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1001,13 +1001,13 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>76</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>4360</v>
+        <v>4364</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>175</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1026,13 +1026,13 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>225</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>4361</v>
+        <v>4365</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1051,13 +1051,13 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>37</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>4362</v>
+        <v>4366</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1076,13 +1076,13 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>37</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>4363</v>
+        <v>4367</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1101,13 +1101,13 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>45</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>4364</v>
+        <v>4368</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>175</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1126,13 +1126,13 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>63</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>4365</v>
+        <v>4369</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1151,13 +1151,13 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>76</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>4366</v>
+        <v>4370</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1176,13 +1176,13 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>77</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>4367</v>
+        <v>4371</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1201,13 +1201,13 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>83</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>4368</v>
+        <v>4372</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>45</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1226,13 +1226,13 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>45</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>4369</v>
+        <v>4373</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>45</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1251,13 +1251,13 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>63</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>4370</v>
+        <v>4374</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>45</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1276,13 +1276,13 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>76</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>4371</v>
+        <v>4375</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>45</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1301,13 +1301,13 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>77</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>4372</v>
+        <v>4376</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>63</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1326,13 +1326,13 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>63</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>4373</v>
+        <v>4377</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>63</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1351,13 +1351,13 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>76</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>4374</v>
+        <v>4378</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>63</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1376,13 +1376,13 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>77</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>4375</v>
+        <v>4379</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>63</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1401,13 +1401,13 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>83</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>4376</v>
+        <v>4380</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1426,13 +1426,13 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>89</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>4377</v>
+        <v>4381</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>76</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1457,7 +1457,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>4378</v>
+        <v>4382</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>76</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1482,7 +1482,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>4379</v>
+        <v>4383</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>76</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1507,7 +1507,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>4380</v>
+        <v>4384</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>76</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1532,7 +1532,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>4381</v>
+        <v>4385</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>77</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1551,13 +1551,13 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>77</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>4382</v>
+        <v>4386</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>77</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1576,13 +1576,13 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>83</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>4383</v>
+        <v>4387</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>83</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1601,13 +1601,13 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>89</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>4384</v>
+        <v>4388</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>89</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1625,106 +1625,6 @@
         </is>
       </c>
       <c r="E48" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>4385</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>MIC19</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>77</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>MIC19</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>77</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>4386</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>MIC19</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>77</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>MIC19</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>83</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>4387</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>MIC19</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>83</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>MIC19</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>4388</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>MIC19</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>MIC19</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
         <is>
           <t>89</t>
         </is>

</xml_diff>